<commit_message>
Reformatação da matriz de requisitos
</commit_message>
<xml_diff>
--- a/DocumentacaoEngenharia/2SIR-ListaRequisitosSIEstacionamento.xlsx
+++ b/DocumentacaoEngenharia/2SIR-ListaRequisitosSIEstacionamento.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Giovanna\Desktop\FIAP\3° SEMESTRE\Business Systems Planning Alalysis e Design\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41FE8EBC-5951-4395-A5F8-C702E3240AA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD9D8D43-A823-4EC5-9957-0A08AF613A84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{31A1ECB0-F9FD-4DA7-8083-81D344CCA4D1}"/>
   </bookViews>
@@ -41,9 +41,6 @@
     <t>LISTA DE REQUISITOS - PROJETO DO SISTEMA DE ESTACIONAMENTO</t>
   </si>
   <si>
-    <t>Nome</t>
-  </si>
-  <si>
     <t>Descrição das regras de domínio</t>
   </si>
   <si>
@@ -52,12 +49,15 @@
   <si>
     <t>*Legenda: Rf = Requisito Funcional; Rnf = Requisito não funcional</t>
   </si>
+  <si>
+    <t>Nome do requisito</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -68,6 +68,21 @@
     <font>
       <sz val="11"/>
       <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="8" tint="-0.499984740745262"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -114,11 +129,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -463,24 +480,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" s="5" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" s="2" t="s">
+      <c r="C4" s="2" t="s">
         <v>1</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Alteralçao da matriz na copia original recuperada
</commit_message>
<xml_diff>
--- a/DocumentacaoEngenharia/2SIR-ListaRequisitosSIEstacionamento.xlsx
+++ b/DocumentacaoEngenharia/2SIR-ListaRequisitosSIEstacionamento.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Giovanna\Desktop\FIAP\3° SEMESTRE\Business Systems Planning Alalysis e Design\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD9D8D43-A823-4EC5-9957-0A08AF613A84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EECA2BE-D823-41F4-B8FC-1FD13931A522}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{31A1ECB0-F9FD-4DA7-8083-81D344CCA4D1}"/>
   </bookViews>
@@ -41,6 +41,9 @@
     <t>LISTA DE REQUISITOS - PROJETO DO SISTEMA DE ESTACIONAMENTO</t>
   </si>
   <si>
+    <t>Nome</t>
+  </si>
+  <si>
     <t>Descrição das regras de domínio</t>
   </si>
   <si>
@@ -49,15 +52,12 @@
   <si>
     <t>*Legenda: Rf = Requisito Funcional; Rnf = Requisito não funcional</t>
   </si>
-  <si>
-    <t>Nome do requisito</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -68,14 +68,6 @@
     <font>
       <sz val="11"/>
       <color theme="0"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -129,13 +121,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -480,24 +471,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="4" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
-        <v>2</v>
-      </c>
       <c r="B4" s="2" t="s">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">

</xml_diff>